<commit_message>
task_2: all 54 forecasts — Country 2 (27) + Country 5 (27)
TI/TN/TG x targets 2/4/6 x Oil 20/50/140 for each country
Country 2: Pi=5.59, R=16, Un=2.2, NAIRU=4.3, Debt 17.85% — emerging
Country 5: Pi=2.63, R=3.63, Un=4.4, NAIRU=4.3, Debt 115.77% — high debt
</commit_message>
<xml_diff>
--- a/results_task_2/deepseek/2_Y_N_TG_2_oil20.xlsx
+++ b/results_task_2/deepseek/2_Y_N_TG_2_oil20.xlsx
@@ -608,7 +608,7 @@
         <v>3.7</v>
       </c>
       <c r="I3" t="n">
-        <v>2.8</v>
+        <v>2.9</v>
       </c>
       <c r="J3" t="n">
         <v>4.3</v>
@@ -670,7 +670,7 @@
         <v>2.5</v>
       </c>
       <c r="I4" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="J4" t="n">
         <v>4.6</v>

</xml_diff>